<commit_message>
Effettuati nuovamente i tests per documento RAD. Modificata la checklist (accreditamento-checklist_V8.2.7.xlsx) e il data.json.
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#GSQUAREDXX/Gsquared/ReSked/6.0/accreditamento-checklist_V8.2.7.xlsx
+++ b/GATEWAY/A1#111#GSQUAREDXX/Gsquared/ReSked/6.0/accreditamento-checklist_V8.2.7.xlsx
@@ -451,10 +451,10 @@
     <t xml:space="preserve">VALIDAZIONE_TOKEN_JWT_RAD_KO</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-01-23T16:49:11.000000Z </t>
-  </si>
-  <si>
-    <t xml:space="preserve">bade912c757398a09e66f857e5b645e3</t>
+    <t xml:space="preserve">2026-03-02T08:50:07.000000Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">46e243df4ddc1e29716b9ec0b0d514d9</t>
   </si>
   <si>
     <t xml:space="preserve">SI</t>
@@ -561,10 +561,10 @@
     <t xml:space="preserve">VALIDAZIONE_TOKEN_JWT_CAMPO_RAD_KO</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-01-23T16:49:26.000000Z </t>
-  </si>
-  <si>
-    <t xml:space="preserve">2e9c0f816dd72ec4043a1a1dd2fe90a8 </t>
+    <t xml:space="preserve">2026-03-02T08:53:00.000000Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">74b9c4a54948444cb7c5d38d0b58c670</t>
   </si>
   <si>
     <t xml:space="preserve">Errore durante la richiesta di validazione: Campo token JWT non valido.  Il campo action_id non è corretto </t>
@@ -765,13 +765,13 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 8" riportata nei documenti "casi di test RAD" e "CDA2_Referto_di_Radiologia_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-01-26T09:40:51.000000Z </t>
-  </si>
-  <si>
-    <t xml:space="preserve">be9eee13c77315d7030d510874e61047 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.16.840.1.113883.2.9.2.120.4.4.ea747adf46c3de160cac31bc9288936669afb363d886e4f5019d174bc64851ce.49688150ec^^^^urn:ihe:iti:xdw:2013:workflowInstanceId </t>
+    <t xml:space="preserve">2026-03-02T08:41:31.000000Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6d0182e108d9b8953836bd31772b1d7e</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.16.840.1.113883.2.9.2.120.4.4.a203546e0ed4a5b969e5ab5573634ab9e74f3e25efd819448c4f9dc023b85b68.6c86ba00d9^^^^urn:ihe:iti:xdw:2013:workflowInstanceId </t>
   </si>
   <si>
     <t xml:space="preserve">Errore nel CDA. Errore semantico. [ERRORE-11| L'elemento ClinicalDocument/recordTarget/patientRole/addr DEVE riportare i suoi sotto-elementi 'country', 'city' e 'streetAddressLine'.   ] </t>
@@ -780,13 +780,13 @@
     <t xml:space="preserve">VALIDAZIONE_CDA2_RAD_CT9_KO</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-01-26T09:46:23.000000Z </t>
-  </si>
-  <si>
-    <t xml:space="preserve">b3fc336b054fd5d811fbabf85bdfa617</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.16.840.1.113883.2.9.2.120.4.4.d02d54208bc8f4b8cf90d549115b59cfbd756236730d67c5e7c81bb95ce2e382.84dda68a1b^^^^urn:ihe:iti:xdw:2013:workflowInstanceId </t>
+    <t xml:space="preserve">2026-03-02T08:56:09.000000Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">379ee3863a35500a668c77b473dc8655</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.16.840.1.113883.2.9.2.120.4.4.3907349ab97c8aa5d585cd04c5b713da8e40ad4ae45c76ccf983bab03e54db0c.f31c6149d5^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
     <t xml:space="preserve">Errore nel CDA. Errore semantico. [ERRORE-14| L'elemento ClinicalDocument/recordTaget/patientRole/patient/name DEVE riportare gli elementi 'given' e 'family']</t>
@@ -813,13 +813,13 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 13" riportata nei documenti "casi di test RAD" e "CDA2_Referto_di_Radiologia_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-01-26T09:52:30.000000Z </t>
-  </si>
-  <si>
-    <t xml:space="preserve">5359b804e0393254881575c99799c930 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.16.840.1.113883.2.9.2.120.4.4.77ca0c34883c900041e5dcf393913f54331d458e4e4a45d2f56f048d6227b7ca.df503f5aed^^^^urn:ihe:iti:xdw:2013:workflowInstanceId </t>
+    <t xml:space="preserve">2026-03-02T09:19:49.000000Z </t>
+  </si>
+  <si>
+    <t xml:space="preserve">908e54a665c7400c99e108b3f98a3f67</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.16.840.1.113883.2.9.2.120.4.4.eb3d0ef8d6548e435658a84e35addf328558bd0f444454b8fbd17bc2cefa2445.c80ddd3a1d^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
     <t xml:space="preserve">Errore nel CDA. Errore di sintassi. ERROR: -1,-1 cvc-complex-type.2.4.b: The content of element 'order' is not complete. One of '{\"urn:hl7-org:v3\":realmCode, \"urn:hl7-org:v3\":typeId, \"urn:hl7-org:v3\":templateId, \"urn:hl7-org:v3\":id}' is expected. </t>
@@ -852,13 +852,13 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 16" riportata nei documenti "casi di test RAD" e "CDA2_Referto_di_Radiologia_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-01-26T09:56:15.000000Z </t>
-  </si>
-  <si>
-    <t xml:space="preserve">6bc30a339318792c205497da31ac737e </t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.16.840.1.113883.2.9.2.120.4.4.189a1b8b3270cbfb044f533974be40172e1ce650542fd4c62bdc19201a084310.b78ee5ba8e^^^^urn:ihe:iti:xdw:2013:workflowInstanceId </t>
+    <t xml:space="preserve">2026-03-02T09:27:46.000000Z </t>
+  </si>
+  <si>
+    <t xml:space="preserve">7372df6265f65fee8726f2359d6b8698 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.16.840.1.113883.2.9.2.120.4.4.99c141d80f222319a371d1a71aeacc05598902a1350cebdae2b3874868f5e80e.3e1d6eab4e^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
     <t xml:space="preserve">Errore nel CDA. Errore semantico. [ERRORE-b13| Sezione Precedenti Esami Eseguiti: La section deve contenere l'elemento 'text'.]</t>
@@ -906,13 +906,13 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 22" riportata nei documenti "casi di test RAD" e "CDA2_Referto_di_Radiologia_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-01-26T10:01:20.000000Z </t>
-  </si>
-  <si>
-    <t xml:space="preserve">a32c6c7f007372a85f366fb5dffd0354 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.16.840.1.113883.2.9.2.120.4.4.76039f59c3cc484a467700dd14b75fa3fd94e7bb46d64d0d41d9a8b441beffdf.89b3b6321f^^^^urn:ihe:iti:xdw:2013:workflowInstanceId </t>
+    <t xml:space="preserve">2026-03-02T09:40:23.000000Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8feec1e7dd24b46943e0bc364848574 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.16.840.1.113883.2.9.2.120.4.4.c4cd94b898edd41bcaeb38b2a2f5dad6dc446af6fbee1843ac6e9ff126285d58.02b4d7f8e8^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
     <t xml:space="preserve">Errore nel CDA. Errore terminologico. Almeno uno dei seguenti vocaboli non è censito: [CodeSystem: 2.16.840.1.113883.6.103, Codes: 666.6] </t>
@@ -1874,13 +1874,13 @@
 I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso nella sezione "CASO DI TEST 24" riportata nei documenti "casi di test RAD" e "CDA2_Referto_di_Radiologia_KO" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-01-26T10:13:58.000000Z </t>
-  </si>
-  <si>
-    <t xml:space="preserve">05bce399a7dd647fd8575b1e0a60d4a4 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.16.840.1.113883.2.9.2.120.4.4.d08a605c7b511afb6e0a0c99027ee9c12182c0194128a0b7296f614b251edead.09722edbe2^^^^urn:ihe:iti:xdw:2013:workflowInstanceId </t>
+    <t xml:space="preserve">2026-03-02T10:06:24.000000Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2fb44d677815619d658cc8ce4822350b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.16.840.1.113883.2.9.2.120.4.4.366e96c85937781827d1355f4a625bbeb7a1f037935a6cd67b5ba3f113016ca0.52a6ea300a^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
     <t xml:space="preserve">Errore nel CDA. Errore di sintassi. ERROR: -1,-1 cvc-complex-type.2.4.a: Invalid content was found starting with element '{\"urn:hl7-org:v3\":languageCode}'. One of '{\"urn:hl7-org:v3\":confidentialityCode}' is expected. </t>
@@ -1961,13 +1961,13 @@
 Il Documento CDA2 Referto Radiologia dovrà essere composto in modo da risultare valido dal punto di vista sintattico, semantico, terminologico. I dati utilizzati per comporre il CDA2 dovranno essere conformi alle section e le entry secondo quanto espresso dalla sezione "CASO DI TEST 25" riportata nei documenti "casi di test RAD" e "CDA2_Referto_di_Radiologia_OK" presenti al path https://github.com/ministero-salute/it-fse-accreditamento.</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-02-05T16:45:16.000000Z </t>
-  </si>
-  <si>
-    <t xml:space="preserve">6a2637346a46f3eed9087b2337ad9f64</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.16.840.1.113883.2.9.2.120.4.4.068903c591f88636d4e4d57ea4e5ebdd2ca921580ea8de264d7ced19993d71d1.845540672a^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+    <t xml:space="preserve">2026-03-02T10:12:08.000000Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">515cd2b5471647ed042ddf82af4b25bd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.16.840.1.113883.2.9.2.120.4.4.ce0442093c76518ef80025c6e0a79f5ee73dca90df17fff3027ea7abe927ca8a.d14b7b7dc7^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
   <si>
     <t xml:space="preserve">VALIDAZIONE_CDA2_RAD_CT26</t>
@@ -2144,7 +2144,7 @@
     <numFmt numFmtId="165" formatCode="@"/>
     <numFmt numFmtId="166" formatCode="d/m/yyyy"/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2257,17 +2257,23 @@
       <family val="1"/>
     </font>
     <font>
-      <sz val="10"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
@@ -2483,7 +2489,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="64">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2648,27 +2654,15 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="166" fontId="15" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="1"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="15" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="1"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="15" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="1"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="166" fontId="16" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="1"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="16" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="1"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2676,20 +2670,36 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="1"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="166" fontId="17" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="1"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="18" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="1"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="18" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="1"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="4" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="17" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="1"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="5" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="15" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="1"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -2700,7 +2710,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="1"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4657,7 +4667,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="89.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="89.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="30" t="n">
         <v>31</v>
       </c>
@@ -4674,12 +4684,12 @@
         <v>53</v>
       </c>
       <c r="F14" s="33" t="n">
-        <v>46045</v>
-      </c>
-      <c r="G14" s="39" t="s">
+        <v>46083</v>
+      </c>
+      <c r="G14" s="41" t="s">
         <v>61</v>
       </c>
-      <c r="H14" s="39" t="s">
+      <c r="H14" s="41" t="s">
         <v>62</v>
       </c>
       <c r="I14" s="39"/>
@@ -4706,7 +4716,7 @@
       <c r="R14" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="S14" s="41" t="s">
+      <c r="S14" s="42" t="s">
         <v>66</v>
       </c>
       <c r="T14" s="34"/>
@@ -4765,7 +4775,7 @@
       <c r="R15" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="S15" s="41" t="s">
+      <c r="S15" s="42" t="s">
         <v>66</v>
       </c>
       <c r="T15" s="34"/>
@@ -4997,7 +5007,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="89.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="89.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="30" t="n">
         <v>39</v>
       </c>
@@ -5014,12 +5024,12 @@
         <v>78</v>
       </c>
       <c r="F22" s="33" t="n">
-        <v>46045</v>
-      </c>
-      <c r="G22" s="39" t="s">
+        <v>46083</v>
+      </c>
+      <c r="G22" s="41" t="s">
         <v>82</v>
       </c>
-      <c r="H22" s="39" t="s">
+      <c r="H22" s="41" t="s">
         <v>83</v>
       </c>
       <c r="I22" s="39"/>
@@ -5046,7 +5056,7 @@
       <c r="R22" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="S22" s="41" t="s">
+      <c r="S22" s="42" t="s">
         <v>66</v>
       </c>
       <c r="T22" s="34"/>
@@ -5105,7 +5115,7 @@
       <c r="R23" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="S23" s="41" t="s">
+      <c r="S23" s="42" t="s">
         <v>66</v>
       </c>
       <c r="T23" s="34"/>
@@ -5343,7 +5353,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="89.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="89.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="30" t="n">
         <v>47</v>
       </c>
@@ -5360,7 +5370,7 @@
         <v>92</v>
       </c>
       <c r="F30" s="33" t="n">
-        <v>46045</v>
+        <v>46083</v>
       </c>
       <c r="G30" s="33"/>
       <c r="H30" s="33"/>
@@ -5388,7 +5398,7 @@
       <c r="R30" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="S30" s="41" t="s">
+      <c r="S30" s="42" t="s">
         <v>97</v>
       </c>
       <c r="T30" s="34"/>
@@ -5443,7 +5453,7 @@
       <c r="R31" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="S31" s="41" t="s">
+      <c r="S31" s="42" t="s">
         <v>97</v>
       </c>
       <c r="T31" s="34"/>
@@ -6236,7 +6246,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="89.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="89.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="30" t="n">
         <v>76</v>
       </c>
@@ -6277,7 +6287,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="89.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="89.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="30" t="n">
         <v>78</v>
       </c>
@@ -6294,15 +6304,15 @@
         <v>142</v>
       </c>
       <c r="F54" s="33" t="n">
-        <v>46048</v>
-      </c>
-      <c r="G54" s="39" t="s">
+        <v>46083</v>
+      </c>
+      <c r="G54" s="41" t="s">
         <v>143</v>
       </c>
-      <c r="H54" s="39" t="s">
+      <c r="H54" s="41" t="s">
         <v>144</v>
       </c>
-      <c r="I54" s="39" t="s">
+      <c r="I54" s="41" t="s">
         <v>145</v>
       </c>
       <c r="J54" s="34" t="s">
@@ -6328,7 +6338,7 @@
       <c r="R54" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="S54" s="41" t="s">
+      <c r="S54" s="42" t="s">
         <v>97</v>
       </c>
       <c r="T54" s="34"/>
@@ -6338,7 +6348,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="89.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="89.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="30" t="n">
         <v>79</v>
       </c>
@@ -6355,7 +6365,7 @@
         <v>142</v>
       </c>
       <c r="F55" s="33" t="n">
-        <v>46048</v>
+        <v>46083</v>
       </c>
       <c r="G55" s="39" t="s">
         <v>148</v>
@@ -6389,7 +6399,7 @@
       <c r="R55" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="S55" s="41" t="s">
+      <c r="S55" s="42" t="s">
         <v>97</v>
       </c>
       <c r="T55" s="34"/>
@@ -6399,7 +6409,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="56" customFormat="false" ht="89.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="56" customFormat="false" ht="89.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="30" t="n">
         <v>80</v>
       </c>
@@ -6439,7 +6449,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="89.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="89.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="30" t="n">
         <v>81</v>
       </c>
@@ -6480,7 +6490,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="89.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="89.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="30" t="n">
         <v>83</v>
       </c>
@@ -6497,15 +6507,15 @@
         <v>157</v>
       </c>
       <c r="F58" s="33" t="n">
-        <v>46048</v>
-      </c>
-      <c r="G58" s="39" t="s">
+        <v>46083</v>
+      </c>
+      <c r="G58" s="41" t="s">
         <v>158</v>
       </c>
-      <c r="H58" s="39" t="s">
+      <c r="H58" s="41" t="s">
         <v>159</v>
       </c>
-      <c r="I58" s="39" t="s">
+      <c r="I58" s="41" t="s">
         <v>160</v>
       </c>
       <c r="J58" s="34" t="s">
@@ -6531,7 +6541,7 @@
       <c r="R58" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="S58" s="41" t="s">
+      <c r="S58" s="42" t="s">
         <v>162</v>
       </c>
       <c r="T58" s="34"/>
@@ -6541,7 +6551,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="89.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="89.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="30" t="n">
         <v>84</v>
       </c>
@@ -6582,7 +6592,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="89.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="89.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="30" t="n">
         <v>85</v>
       </c>
@@ -6623,7 +6633,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="89.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="89.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="30" t="n">
         <v>86</v>
       </c>
@@ -6639,8 +6649,8 @@
       <c r="E61" s="31" t="s">
         <v>169</v>
       </c>
-      <c r="F61" s="33" t="n">
-        <v>46048</v>
+      <c r="F61" s="43" t="n">
+        <v>46083</v>
       </c>
       <c r="G61" s="39" t="s">
         <v>170</v>
@@ -6674,7 +6684,7 @@
       <c r="R61" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="S61" s="41" t="s">
+      <c r="S61" s="42" t="s">
         <v>97</v>
       </c>
       <c r="T61" s="34"/>
@@ -6684,7 +6694,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="89.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="89.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="30" t="n">
         <v>87</v>
       </c>
@@ -6725,7 +6735,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="89.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="63" customFormat="false" ht="89.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="30" t="n">
         <v>88</v>
       </c>
@@ -6766,7 +6776,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="89.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="64" customFormat="false" ht="89.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="30" t="n">
         <v>89</v>
       </c>
@@ -6807,7 +6817,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="89.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="65" customFormat="false" ht="89.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="30" t="n">
         <v>90</v>
       </c>
@@ -6848,7 +6858,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="89.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="66" customFormat="false" ht="89.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="30" t="n">
         <v>91</v>
       </c>
@@ -6889,7 +6899,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="67" customFormat="false" ht="89.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="67" customFormat="false" ht="89.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="30" t="n">
         <v>92</v>
       </c>
@@ -6905,8 +6915,8 @@
       <c r="E67" s="31" t="s">
         <v>185</v>
       </c>
-      <c r="F67" s="33" t="n">
-        <v>46048</v>
+      <c r="F67" s="43" t="n">
+        <v>46083</v>
       </c>
       <c r="G67" s="39" t="s">
         <v>186</v>
@@ -6940,7 +6950,7 @@
       <c r="R67" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="S67" s="41" t="s">
+      <c r="S67" s="42" t="s">
         <v>190</v>
       </c>
       <c r="T67" s="34"/>
@@ -6950,7 +6960,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="89.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="68" customFormat="false" ht="89.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="30" t="n">
         <v>93</v>
       </c>
@@ -8790,13 +8800,13 @@
       <c r="F117" s="33" t="n">
         <v>46077</v>
       </c>
-      <c r="G117" s="42" t="s">
+      <c r="G117" s="44" t="s">
         <v>292</v>
       </c>
-      <c r="H117" s="42" t="s">
+      <c r="H117" s="44" t="s">
         <v>293</v>
       </c>
-      <c r="I117" s="43" t="s">
+      <c r="I117" s="45" t="s">
         <v>294</v>
       </c>
       <c r="J117" s="34" t="s">
@@ -8822,7 +8832,7 @@
       <c r="R117" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="S117" s="41" t="s">
+      <c r="S117" s="42" t="s">
         <v>97</v>
       </c>
       <c r="T117" s="34"/>
@@ -8851,13 +8861,13 @@
       <c r="F118" s="33" t="n">
         <v>46077</v>
       </c>
-      <c r="G118" s="44" t="s">
+      <c r="G118" s="46" t="s">
         <v>298</v>
       </c>
-      <c r="H118" s="44" t="s">
+      <c r="H118" s="46" t="s">
         <v>299</v>
       </c>
-      <c r="I118" s="43" t="s">
+      <c r="I118" s="45" t="s">
         <v>300</v>
       </c>
       <c r="J118" s="34" t="s">
@@ -8871,7 +8881,7 @@
       <c r="N118" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="O118" s="45" t="s">
+      <c r="O118" s="47" t="s">
         <v>301</v>
       </c>
       <c r="P118" s="34" t="s">
@@ -8883,7 +8893,7 @@
       <c r="R118" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="S118" s="41" t="s">
+      <c r="S118" s="42" t="s">
         <v>97</v>
       </c>
       <c r="T118" s="34"/>
@@ -8953,10 +8963,10 @@
       <c r="F120" s="33" t="n">
         <v>46077</v>
       </c>
-      <c r="G120" s="44" t="s">
+      <c r="G120" s="46" t="s">
         <v>306</v>
       </c>
-      <c r="H120" s="44" t="s">
+      <c r="H120" s="46" t="s">
         <v>307</v>
       </c>
       <c r="I120" s="39" t="s">
@@ -8985,7 +8995,7 @@
       <c r="R120" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="S120" s="41" t="s">
+      <c r="S120" s="42" t="s">
         <v>97</v>
       </c>
       <c r="T120" s="34"/>
@@ -9014,13 +9024,13 @@
       <c r="F121" s="33" t="n">
         <v>46077</v>
       </c>
-      <c r="G121" s="42" t="s">
+      <c r="G121" s="44" t="s">
         <v>312</v>
       </c>
-      <c r="H121" s="42" t="s">
+      <c r="H121" s="44" t="s">
         <v>313</v>
       </c>
-      <c r="I121" s="43" t="s">
+      <c r="I121" s="45" t="s">
         <v>314</v>
       </c>
       <c r="J121" s="34" t="s">
@@ -9034,7 +9044,7 @@
       <c r="N121" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="O121" s="45" t="s">
+      <c r="O121" s="47" t="s">
         <v>315</v>
       </c>
       <c r="P121" s="34" t="s">
@@ -9046,7 +9056,7 @@
       <c r="R121" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="S121" s="41" t="s">
+      <c r="S121" s="42" t="s">
         <v>97</v>
       </c>
       <c r="T121" s="34"/>
@@ -9095,7 +9105,7 @@
       <c r="N122" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="O122" s="45" t="s">
+      <c r="O122" s="47" t="s">
         <v>321</v>
       </c>
       <c r="P122" s="34" t="s">
@@ -9107,7 +9117,7 @@
       <c r="R122" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="S122" s="41" t="s">
+      <c r="S122" s="42" t="s">
         <v>97</v>
       </c>
       <c r="T122" s="34"/>
@@ -9136,10 +9146,10 @@
       <c r="F123" s="33" t="n">
         <v>46077</v>
       </c>
-      <c r="G123" s="44" t="s">
+      <c r="G123" s="46" t="s">
         <v>324</v>
       </c>
-      <c r="H123" s="44" t="s">
+      <c r="H123" s="46" t="s">
         <v>325</v>
       </c>
       <c r="I123" s="39" t="s">
@@ -9156,7 +9166,7 @@
       <c r="N123" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="O123" s="45" t="s">
+      <c r="O123" s="47" t="s">
         <v>327</v>
       </c>
       <c r="P123" s="34" t="s">
@@ -9168,7 +9178,7 @@
       <c r="R123" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="S123" s="41" t="s">
+      <c r="S123" s="42" t="s">
         <v>97</v>
       </c>
       <c r="T123" s="34"/>
@@ -9197,7 +9207,7 @@
       <c r="F124" s="33" t="n">
         <v>46077</v>
       </c>
-      <c r="G124" s="44" t="s">
+      <c r="G124" s="46" t="s">
         <v>330</v>
       </c>
       <c r="H124" s="39" t="s">
@@ -9217,7 +9227,7 @@
       <c r="N124" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="O124" s="45" t="s">
+      <c r="O124" s="47" t="s">
         <v>333</v>
       </c>
       <c r="P124" s="34" t="s">
@@ -9229,7 +9239,7 @@
       <c r="R124" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="S124" s="41" t="s">
+      <c r="S124" s="42" t="s">
         <v>97</v>
       </c>
       <c r="T124" s="34"/>
@@ -9258,10 +9268,10 @@
       <c r="F125" s="33" t="n">
         <v>46077</v>
       </c>
-      <c r="G125" s="44" t="s">
+      <c r="G125" s="46" t="s">
         <v>336</v>
       </c>
-      <c r="H125" s="44" t="s">
+      <c r="H125" s="46" t="s">
         <v>337</v>
       </c>
       <c r="I125" s="39" t="s">
@@ -9278,7 +9288,7 @@
       <c r="N125" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="O125" s="45" t="s">
+      <c r="O125" s="47" t="s">
         <v>339</v>
       </c>
       <c r="P125" s="34" t="s">
@@ -9290,7 +9300,7 @@
       <c r="R125" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="S125" s="41" t="s">
+      <c r="S125" s="42" t="s">
         <v>97</v>
       </c>
       <c r="T125" s="34"/>
@@ -9319,13 +9329,13 @@
       <c r="F126" s="33" t="n">
         <v>46077</v>
       </c>
-      <c r="G126" s="44" t="s">
+      <c r="G126" s="46" t="s">
         <v>342</v>
       </c>
-      <c r="H126" s="44" t="s">
+      <c r="H126" s="46" t="s">
         <v>343</v>
       </c>
-      <c r="I126" s="46" t="s">
+      <c r="I126" s="48" t="s">
         <v>344</v>
       </c>
       <c r="J126" s="34" t="s">
@@ -9339,7 +9349,7 @@
       <c r="N126" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="O126" s="45" t="s">
+      <c r="O126" s="47" t="s">
         <v>345</v>
       </c>
       <c r="P126" s="34" t="s">
@@ -9351,7 +9361,7 @@
       <c r="R126" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="S126" s="41" t="s">
+      <c r="S126" s="42" t="s">
         <v>97</v>
       </c>
       <c r="T126" s="34"/>
@@ -9380,13 +9390,13 @@
       <c r="F127" s="33" t="n">
         <v>46077</v>
       </c>
-      <c r="G127" s="44" t="s">
+      <c r="G127" s="46" t="s">
         <v>348</v>
       </c>
-      <c r="H127" s="44" t="s">
+      <c r="H127" s="46" t="s">
         <v>349</v>
       </c>
-      <c r="I127" s="46" t="s">
+      <c r="I127" s="48" t="s">
         <v>350</v>
       </c>
       <c r="J127" s="34" t="s">
@@ -9412,7 +9422,7 @@
       <c r="R127" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="S127" s="41" t="s">
+      <c r="S127" s="42" t="s">
         <v>97</v>
       </c>
       <c r="T127" s="34"/>
@@ -9441,13 +9451,13 @@
       <c r="F128" s="33" t="n">
         <v>46077</v>
       </c>
-      <c r="G128" s="44" t="s">
+      <c r="G128" s="46" t="s">
         <v>354</v>
       </c>
-      <c r="H128" s="44" t="s">
+      <c r="H128" s="46" t="s">
         <v>355</v>
       </c>
-      <c r="I128" s="46" t="s">
+      <c r="I128" s="48" t="s">
         <v>356</v>
       </c>
       <c r="J128" s="34" t="s">
@@ -9473,7 +9483,7 @@
       <c r="R128" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="S128" s="41" t="s">
+      <c r="S128" s="42" t="s">
         <v>97</v>
       </c>
       <c r="T128" s="34"/>
@@ -9502,13 +9512,13 @@
       <c r="F129" s="33" t="n">
         <v>46077</v>
       </c>
-      <c r="G129" s="44" t="s">
+      <c r="G129" s="46" t="s">
         <v>360</v>
       </c>
-      <c r="H129" s="44" t="s">
+      <c r="H129" s="46" t="s">
         <v>361</v>
       </c>
-      <c r="I129" s="46" t="s">
+      <c r="I129" s="48" t="s">
         <v>362</v>
       </c>
       <c r="J129" s="34" t="s">
@@ -9534,7 +9544,7 @@
       <c r="R129" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="S129" s="41" t="s">
+      <c r="S129" s="42" t="s">
         <v>97</v>
       </c>
       <c r="T129" s="34"/>
@@ -9563,10 +9573,10 @@
       <c r="F130" s="33" t="n">
         <v>46077</v>
       </c>
-      <c r="G130" s="47" t="s">
+      <c r="G130" s="44" t="s">
         <v>366</v>
       </c>
-      <c r="H130" s="47" t="s">
+      <c r="H130" s="44" t="s">
         <v>367</v>
       </c>
       <c r="I130" s="39" t="s">
@@ -9583,7 +9593,7 @@
       <c r="N130" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="O130" s="45" t="s">
+      <c r="O130" s="47" t="s">
         <v>369</v>
       </c>
       <c r="P130" s="34" t="s">
@@ -9595,7 +9605,7 @@
       <c r="R130" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="S130" s="41" t="s">
+      <c r="S130" s="42" t="s">
         <v>97</v>
       </c>
       <c r="T130" s="34"/>
@@ -10833,7 +10843,7 @@
       <c r="B164" s="30" t="s">
         <v>47</v>
       </c>
-      <c r="C164" s="48" t="s">
+      <c r="C164" s="49" t="s">
         <v>67</v>
       </c>
       <c r="D164" s="30" t="s">
@@ -10845,13 +10855,13 @@
       <c r="F164" s="33" t="n">
         <v>46077</v>
       </c>
-      <c r="G164" s="47" t="s">
+      <c r="G164" s="44" t="s">
         <v>437</v>
       </c>
-      <c r="H164" s="47" t="s">
+      <c r="H164" s="44" t="s">
         <v>438</v>
       </c>
-      <c r="I164" s="49" t="s">
+      <c r="I164" s="45" t="s">
         <v>439</v>
       </c>
       <c r="J164" s="34" t="s">
@@ -11335,7 +11345,7 @@
       <c r="R176" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="S176" s="41" t="s">
+      <c r="S176" s="42" t="s">
         <v>97</v>
       </c>
       <c r="T176" s="34"/>
@@ -11345,7 +11355,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="177" customFormat="false" ht="89.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="177" customFormat="false" ht="89.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A177" s="30" t="n">
         <v>462</v>
       </c>
@@ -11361,8 +11371,8 @@
       <c r="E177" s="31" t="s">
         <v>470</v>
       </c>
-      <c r="F177" s="33" t="n">
-        <v>46048</v>
+      <c r="F177" s="43" t="n">
+        <v>46083</v>
       </c>
       <c r="G177" s="33" t="s">
         <v>471</v>
@@ -11396,7 +11406,7 @@
       <c r="R177" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="S177" s="41" t="s">
+      <c r="S177" s="42" t="s">
         <v>190</v>
       </c>
       <c r="T177" s="34"/>
@@ -11613,10 +11623,10 @@
       <c r="G183" s="50" t="s">
         <v>487</v>
       </c>
-      <c r="H183" s="44" t="s">
+      <c r="H183" s="46" t="s">
         <v>488</v>
       </c>
-      <c r="I183" s="46" t="s">
+      <c r="I183" s="48" t="s">
         <v>489</v>
       </c>
       <c r="J183" s="34" t="s">
@@ -11642,7 +11652,7 @@
       <c r="R183" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="S183" s="41" t="s">
+      <c r="S183" s="42" t="s">
         <v>97</v>
       </c>
       <c r="T183" s="34"/>
@@ -11726,7 +11736,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="186" s="1" customFormat="true" ht="89.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="186" s="1" customFormat="true" ht="89.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A186" s="30" t="n">
         <v>471</v>
       </c>
@@ -11742,16 +11752,16 @@
       <c r="E186" s="31" t="s">
         <v>496</v>
       </c>
-      <c r="F186" s="39" t="n">
-        <v>46058</v>
-      </c>
-      <c r="G186" s="33" t="s">
+      <c r="F186" s="43" t="n">
+        <v>46083</v>
+      </c>
+      <c r="G186" s="52" t="s">
         <v>497</v>
       </c>
-      <c r="H186" s="33" t="s">
+      <c r="H186" s="52" t="s">
         <v>498</v>
       </c>
-      <c r="I186" s="39" t="s">
+      <c r="I186" s="41" t="s">
         <v>499</v>
       </c>
       <c r="J186" s="34" t="s">
@@ -11773,7 +11783,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="187" s="1" customFormat="true" ht="89.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="187" s="1" customFormat="true" ht="89.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A187" s="30" t="n">
         <v>472</v>
       </c>
@@ -11853,7 +11863,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="189" customFormat="false" ht="89.25" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="189" customFormat="false" ht="89.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A189" s="30" t="n">
         <v>474</v>
       </c>
@@ -11945,7 +11955,7 @@
       <c r="R190" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="S190" s="41" t="s">
+      <c r="S190" s="42" t="s">
         <v>97</v>
       </c>
       <c r="T190" s="34"/>
@@ -12042,7 +12052,7 @@
       <c r="D193" s="30" t="s">
         <v>518</v>
       </c>
-      <c r="E193" s="52" t="s">
+      <c r="E193" s="53" t="s">
         <v>519</v>
       </c>
       <c r="F193" s="33"/>
@@ -16026,6 +16036,7 @@
   <autoFilter ref="A9:W193">
     <filterColumn colId="2">
       <filters>
+        <filter val="RAD"/>
         <filter val="RSA"/>
       </filters>
     </filterColumn>
@@ -16147,7 +16158,7 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="53" t="s">
+      <c r="A1" s="54" t="s">
         <v>523</v>
       </c>
       <c r="B1" s="19" t="s">
@@ -16159,158 +16170,158 @@
       <c r="D1" s="19" t="s">
         <v>525</v>
       </c>
-      <c r="F1" s="54" t="s">
+      <c r="F1" s="55" t="s">
         <v>526</v>
       </c>
-      <c r="G1" s="55" t="s">
+      <c r="G1" s="56" t="s">
         <v>527</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="56" t="s">
+      <c r="A2" s="57" t="s">
         <v>48</v>
       </c>
-      <c r="B2" s="56" t="s">
+      <c r="B2" s="57" t="s">
         <v>528</v>
       </c>
-      <c r="C2" s="57" t="s">
+      <c r="C2" s="58" t="s">
         <v>529</v>
       </c>
-      <c r="D2" s="58" t="s">
+      <c r="D2" s="59" t="s">
         <v>530</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="56" t="s">
+      <c r="A3" s="57" t="s">
         <v>55</v>
       </c>
-      <c r="B3" s="56" t="s">
+      <c r="B3" s="57" t="s">
         <v>528</v>
       </c>
-      <c r="C3" s="57" t="s">
+      <c r="C3" s="58" t="s">
         <v>531</v>
       </c>
-      <c r="D3" s="58" t="s">
+      <c r="D3" s="59" t="s">
         <v>532</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="56" t="s">
+      <c r="A4" s="57" t="s">
         <v>59</v>
       </c>
-      <c r="B4" s="56" t="s">
+      <c r="B4" s="57" t="s">
         <v>528</v>
       </c>
-      <c r="C4" s="57" t="s">
+      <c r="C4" s="58" t="s">
         <v>533</v>
       </c>
-      <c r="D4" s="59" t="s">
+      <c r="D4" s="60" t="s">
         <v>534</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="56" t="s">
+      <c r="A5" s="57" t="s">
         <v>71</v>
       </c>
-      <c r="B5" s="56" t="s">
+      <c r="B5" s="57" t="s">
         <v>528</v>
       </c>
-      <c r="C5" s="57" t="s">
+      <c r="C5" s="58" t="s">
         <v>535</v>
       </c>
-      <c r="D5" s="58" t="s">
+      <c r="D5" s="59" t="s">
         <v>536</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="56" t="s">
+      <c r="A6" s="57" t="s">
         <v>73</v>
       </c>
-      <c r="B6" s="56" t="s">
+      <c r="B6" s="57" t="s">
         <v>528</v>
       </c>
-      <c r="C6" s="57" t="s">
+      <c r="C6" s="58" t="s">
         <v>537</v>
       </c>
-      <c r="D6" s="59" t="s">
+      <c r="D6" s="60" t="s">
         <v>538</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="56" t="s">
+      <c r="A7" s="57" t="s">
         <v>75</v>
       </c>
-      <c r="B7" s="56" t="s">
+      <c r="B7" s="57" t="s">
         <v>528</v>
       </c>
-      <c r="C7" s="57" t="s">
+      <c r="C7" s="58" t="s">
         <v>539</v>
       </c>
-      <c r="D7" s="59" t="s">
+      <c r="D7" s="60" t="s">
         <v>540</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="56" t="s">
+      <c r="A8" s="57" t="s">
         <v>67</v>
       </c>
-      <c r="B8" s="56" t="s">
+      <c r="B8" s="57" t="s">
         <v>528</v>
       </c>
-      <c r="C8" s="57" t="s">
+      <c r="C8" s="58" t="s">
         <v>541</v>
       </c>
-      <c r="D8" s="59" t="s">
+      <c r="D8" s="60" t="s">
         <v>542</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="56" t="s">
+      <c r="A9" s="57" t="s">
         <v>57</v>
       </c>
-      <c r="B9" s="56" t="s">
+      <c r="B9" s="57" t="s">
         <v>528</v>
       </c>
-      <c r="C9" s="57" t="s">
+      <c r="C9" s="58" t="s">
         <v>543</v>
       </c>
-      <c r="D9" s="59" t="s">
+      <c r="D9" s="60" t="s">
         <v>544</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="36.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="56" t="s">
+      <c r="A10" s="57" t="s">
         <v>545</v>
       </c>
-      <c r="B10" s="56" t="s">
+      <c r="B10" s="57" t="s">
         <v>528</v>
       </c>
-      <c r="C10" s="60" t="s">
+      <c r="C10" s="61" t="s">
         <v>546</v>
       </c>
-      <c r="D10" s="58" t="s">
+      <c r="D10" s="59" t="s">
         <v>547</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="56" t="s">
+      <c r="A11" s="57" t="s">
         <v>404</v>
       </c>
-      <c r="B11" s="56" t="s">
+      <c r="B11" s="57" t="s">
         <v>528</v>
       </c>
-      <c r="C11" s="57" t="s">
+      <c r="C11" s="58" t="s">
         <v>548</v>
       </c>
-      <c r="D11" s="59" t="s">
+      <c r="D11" s="60" t="s">
         <v>549</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D12" s="61"/>
+      <c r="D12" s="62"/>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D13" s="61"/>
+      <c r="D13" s="62"/>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -17286,32 +17297,32 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="62" t="s">
+      <c r="A1" s="63" t="s">
         <v>43</v>
       </c>
-      <c r="B1" s="62" t="s">
+      <c r="B1" s="63" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="62" t="s">
+      <c r="A2" s="63" t="s">
         <v>550</v>
       </c>
-      <c r="B2" s="62" t="s">
+      <c r="B2" s="63" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="62" t="s">
+      <c r="A3" s="63" t="s">
         <v>551</v>
       </c>
-      <c r="B3" s="62" t="s">
+      <c r="B3" s="63" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="62"/>
-      <c r="B4" s="62"/>
+      <c r="A4" s="63"/>
+      <c r="B4" s="63"/>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
Apportata modifica a colonna P della checklist per i test 31, 32, 39, 40 coerentemente con quanto dichiarato in colonna S.
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#GSQUAREDXX/Gsquared/ReSked/6.0/accreditamento-checklist_V8.2.7.xlsx
+++ b/GATEWAY/A1#111#GSQUAREDXX/Gsquared/ReSked/6.0/accreditamento-checklist_V8.2.7.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
@@ -2144,7 +2144,7 @@
     <numFmt numFmtId="165" formatCode="@"/>
     <numFmt numFmtId="166" formatCode="d/m/yyyy"/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="19">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2249,18 +2249,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -2489,7 +2477,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="61">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2662,27 +2650,19 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="166" fontId="15" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="1"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="166" fontId="16" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="1"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="17" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="1"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="17" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="1"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="18" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="1"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="18" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="16" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="1"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2690,16 +2670,12 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="5" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="15" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="1"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -2710,7 +2686,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false" readingOrder="1"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4708,7 +4684,7 @@
         <v>64</v>
       </c>
       <c r="P14" s="34" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="Q14" s="34" t="s">
         <v>65</v>
@@ -4767,7 +4743,7 @@
         <v>64</v>
       </c>
       <c r="P15" s="34" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="Q15" s="34" t="s">
         <v>65</v>
@@ -5048,7 +5024,7 @@
         <v>84</v>
       </c>
       <c r="P22" s="34" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="Q22" s="34" t="s">
         <v>65</v>
@@ -5107,7 +5083,7 @@
         <v>84</v>
       </c>
       <c r="P23" s="34" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="Q23" s="34" t="s">
         <v>65</v>
@@ -6649,7 +6625,7 @@
       <c r="E61" s="31" t="s">
         <v>169</v>
       </c>
-      <c r="F61" s="43" t="n">
+      <c r="F61" s="33" t="n">
         <v>46083</v>
       </c>
       <c r="G61" s="39" t="s">
@@ -6915,7 +6891,7 @@
       <c r="E67" s="31" t="s">
         <v>185</v>
       </c>
-      <c r="F67" s="43" t="n">
+      <c r="F67" s="33" t="n">
         <v>46083</v>
       </c>
       <c r="G67" s="39" t="s">
@@ -8800,13 +8776,13 @@
       <c r="F117" s="33" t="n">
         <v>46077</v>
       </c>
-      <c r="G117" s="44" t="s">
+      <c r="G117" s="43" t="s">
         <v>292</v>
       </c>
-      <c r="H117" s="44" t="s">
+      <c r="H117" s="43" t="s">
         <v>293</v>
       </c>
-      <c r="I117" s="45" t="s">
+      <c r="I117" s="41" t="s">
         <v>294</v>
       </c>
       <c r="J117" s="34" t="s">
@@ -8861,13 +8837,13 @@
       <c r="F118" s="33" t="n">
         <v>46077</v>
       </c>
-      <c r="G118" s="46" t="s">
+      <c r="G118" s="44" t="s">
         <v>298</v>
       </c>
-      <c r="H118" s="46" t="s">
+      <c r="H118" s="44" t="s">
         <v>299</v>
       </c>
-      <c r="I118" s="45" t="s">
+      <c r="I118" s="41" t="s">
         <v>300</v>
       </c>
       <c r="J118" s="34" t="s">
@@ -8881,7 +8857,7 @@
       <c r="N118" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="O118" s="47" t="s">
+      <c r="O118" s="45" t="s">
         <v>301</v>
       </c>
       <c r="P118" s="34" t="s">
@@ -8963,10 +8939,10 @@
       <c r="F120" s="33" t="n">
         <v>46077</v>
       </c>
-      <c r="G120" s="46" t="s">
+      <c r="G120" s="44" t="s">
         <v>306</v>
       </c>
-      <c r="H120" s="46" t="s">
+      <c r="H120" s="44" t="s">
         <v>307</v>
       </c>
       <c r="I120" s="39" t="s">
@@ -9024,13 +9000,13 @@
       <c r="F121" s="33" t="n">
         <v>46077</v>
       </c>
-      <c r="G121" s="44" t="s">
+      <c r="G121" s="43" t="s">
         <v>312</v>
       </c>
-      <c r="H121" s="44" t="s">
+      <c r="H121" s="43" t="s">
         <v>313</v>
       </c>
-      <c r="I121" s="45" t="s">
+      <c r="I121" s="41" t="s">
         <v>314</v>
       </c>
       <c r="J121" s="34" t="s">
@@ -9044,7 +9020,7 @@
       <c r="N121" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="O121" s="47" t="s">
+      <c r="O121" s="45" t="s">
         <v>315</v>
       </c>
       <c r="P121" s="34" t="s">
@@ -9105,7 +9081,7 @@
       <c r="N122" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="O122" s="47" t="s">
+      <c r="O122" s="45" t="s">
         <v>321</v>
       </c>
       <c r="P122" s="34" t="s">
@@ -9146,10 +9122,10 @@
       <c r="F123" s="33" t="n">
         <v>46077</v>
       </c>
-      <c r="G123" s="46" t="s">
+      <c r="G123" s="44" t="s">
         <v>324</v>
       </c>
-      <c r="H123" s="46" t="s">
+      <c r="H123" s="44" t="s">
         <v>325</v>
       </c>
       <c r="I123" s="39" t="s">
@@ -9166,7 +9142,7 @@
       <c r="N123" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="O123" s="47" t="s">
+      <c r="O123" s="45" t="s">
         <v>327</v>
       </c>
       <c r="P123" s="34" t="s">
@@ -9207,7 +9183,7 @@
       <c r="F124" s="33" t="n">
         <v>46077</v>
       </c>
-      <c r="G124" s="46" t="s">
+      <c r="G124" s="44" t="s">
         <v>330</v>
       </c>
       <c r="H124" s="39" t="s">
@@ -9227,7 +9203,7 @@
       <c r="N124" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="O124" s="47" t="s">
+      <c r="O124" s="45" t="s">
         <v>333</v>
       </c>
       <c r="P124" s="34" t="s">
@@ -9268,10 +9244,10 @@
       <c r="F125" s="33" t="n">
         <v>46077</v>
       </c>
-      <c r="G125" s="46" t="s">
+      <c r="G125" s="44" t="s">
         <v>336</v>
       </c>
-      <c r="H125" s="46" t="s">
+      <c r="H125" s="44" t="s">
         <v>337</v>
       </c>
       <c r="I125" s="39" t="s">
@@ -9288,7 +9264,7 @@
       <c r="N125" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="O125" s="47" t="s">
+      <c r="O125" s="45" t="s">
         <v>339</v>
       </c>
       <c r="P125" s="34" t="s">
@@ -9329,13 +9305,13 @@
       <c r="F126" s="33" t="n">
         <v>46077</v>
       </c>
-      <c r="G126" s="46" t="s">
+      <c r="G126" s="44" t="s">
         <v>342</v>
       </c>
-      <c r="H126" s="46" t="s">
+      <c r="H126" s="44" t="s">
         <v>343</v>
       </c>
-      <c r="I126" s="48" t="s">
+      <c r="I126" s="46" t="s">
         <v>344</v>
       </c>
       <c r="J126" s="34" t="s">
@@ -9349,7 +9325,7 @@
       <c r="N126" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="O126" s="47" t="s">
+      <c r="O126" s="45" t="s">
         <v>345</v>
       </c>
       <c r="P126" s="34" t="s">
@@ -9390,13 +9366,13 @@
       <c r="F127" s="33" t="n">
         <v>46077</v>
       </c>
-      <c r="G127" s="46" t="s">
+      <c r="G127" s="44" t="s">
         <v>348</v>
       </c>
-      <c r="H127" s="46" t="s">
+      <c r="H127" s="44" t="s">
         <v>349</v>
       </c>
-      <c r="I127" s="48" t="s">
+      <c r="I127" s="46" t="s">
         <v>350</v>
       </c>
       <c r="J127" s="34" t="s">
@@ -9451,13 +9427,13 @@
       <c r="F128" s="33" t="n">
         <v>46077</v>
       </c>
-      <c r="G128" s="46" t="s">
+      <c r="G128" s="44" t="s">
         <v>354</v>
       </c>
-      <c r="H128" s="46" t="s">
+      <c r="H128" s="44" t="s">
         <v>355</v>
       </c>
-      <c r="I128" s="48" t="s">
+      <c r="I128" s="46" t="s">
         <v>356</v>
       </c>
       <c r="J128" s="34" t="s">
@@ -9512,13 +9488,13 @@
       <c r="F129" s="33" t="n">
         <v>46077</v>
       </c>
-      <c r="G129" s="46" t="s">
+      <c r="G129" s="44" t="s">
         <v>360</v>
       </c>
-      <c r="H129" s="46" t="s">
+      <c r="H129" s="44" t="s">
         <v>361</v>
       </c>
-      <c r="I129" s="48" t="s">
+      <c r="I129" s="46" t="s">
         <v>362</v>
       </c>
       <c r="J129" s="34" t="s">
@@ -9573,10 +9549,10 @@
       <c r="F130" s="33" t="n">
         <v>46077</v>
       </c>
-      <c r="G130" s="44" t="s">
+      <c r="G130" s="43" t="s">
         <v>366</v>
       </c>
-      <c r="H130" s="44" t="s">
+      <c r="H130" s="43" t="s">
         <v>367</v>
       </c>
       <c r="I130" s="39" t="s">
@@ -9593,7 +9569,7 @@
       <c r="N130" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="O130" s="47" t="s">
+      <c r="O130" s="45" t="s">
         <v>369</v>
       </c>
       <c r="P130" s="34" t="s">
@@ -10843,7 +10819,7 @@
       <c r="B164" s="30" t="s">
         <v>47</v>
       </c>
-      <c r="C164" s="49" t="s">
+      <c r="C164" s="47" t="s">
         <v>67</v>
       </c>
       <c r="D164" s="30" t="s">
@@ -10855,13 +10831,13 @@
       <c r="F164" s="33" t="n">
         <v>46077</v>
       </c>
-      <c r="G164" s="44" t="s">
+      <c r="G164" s="43" t="s">
         <v>437</v>
       </c>
-      <c r="H164" s="44" t="s">
+      <c r="H164" s="43" t="s">
         <v>438</v>
       </c>
-      <c r="I164" s="45" t="s">
+      <c r="I164" s="41" t="s">
         <v>439</v>
       </c>
       <c r="J164" s="34" t="s">
@@ -11313,7 +11289,7 @@
       <c r="F176" s="33" t="n">
         <v>46077</v>
       </c>
-      <c r="G176" s="50" t="s">
+      <c r="G176" s="48" t="s">
         <v>465</v>
       </c>
       <c r="H176" s="33" t="s">
@@ -11371,7 +11347,7 @@
       <c r="E177" s="31" t="s">
         <v>470</v>
       </c>
-      <c r="F177" s="43" t="n">
+      <c r="F177" s="33" t="n">
         <v>46083</v>
       </c>
       <c r="G177" s="33" t="s">
@@ -11620,13 +11596,13 @@
       <c r="F183" s="33" t="n">
         <v>46077</v>
       </c>
-      <c r="G183" s="50" t="s">
+      <c r="G183" s="48" t="s">
         <v>487</v>
       </c>
-      <c r="H183" s="46" t="s">
+      <c r="H183" s="44" t="s">
         <v>488</v>
       </c>
-      <c r="I183" s="48" t="s">
+      <c r="I183" s="46" t="s">
         <v>489</v>
       </c>
       <c r="J183" s="34" t="s">
@@ -11743,7 +11719,7 @@
       <c r="B186" s="30" t="s">
         <v>47</v>
       </c>
-      <c r="C186" s="51" t="s">
+      <c r="C186" s="49" t="s">
         <v>59</v>
       </c>
       <c r="D186" s="30" t="s">
@@ -11752,13 +11728,13 @@
       <c r="E186" s="31" t="s">
         <v>496</v>
       </c>
-      <c r="F186" s="43" t="n">
+      <c r="F186" s="33" t="n">
         <v>46083</v>
       </c>
-      <c r="G186" s="52" t="s">
+      <c r="G186" s="43" t="s">
         <v>497</v>
       </c>
-      <c r="H186" s="52" t="s">
+      <c r="H186" s="43" t="s">
         <v>498</v>
       </c>
       <c r="I186" s="41" t="s">
@@ -12052,7 +12028,7 @@
       <c r="D193" s="30" t="s">
         <v>518</v>
       </c>
-      <c r="E193" s="53" t="s">
+      <c r="E193" s="50" t="s">
         <v>519</v>
       </c>
       <c r="F193" s="33"/>
@@ -16158,7 +16134,7 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="51" t="s">
         <v>523</v>
       </c>
       <c r="B1" s="19" t="s">
@@ -16170,158 +16146,158 @@
       <c r="D1" s="19" t="s">
         <v>525</v>
       </c>
-      <c r="F1" s="55" t="s">
+      <c r="F1" s="52" t="s">
         <v>526</v>
       </c>
-      <c r="G1" s="56" t="s">
+      <c r="G1" s="53" t="s">
         <v>527</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="57" t="s">
+      <c r="A2" s="54" t="s">
         <v>48</v>
       </c>
-      <c r="B2" s="57" t="s">
+      <c r="B2" s="54" t="s">
         <v>528</v>
       </c>
-      <c r="C2" s="58" t="s">
+      <c r="C2" s="55" t="s">
         <v>529</v>
       </c>
-      <c r="D2" s="59" t="s">
+      <c r="D2" s="56" t="s">
         <v>530</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="57" t="s">
+      <c r="A3" s="54" t="s">
         <v>55</v>
       </c>
-      <c r="B3" s="57" t="s">
+      <c r="B3" s="54" t="s">
         <v>528</v>
       </c>
-      <c r="C3" s="58" t="s">
+      <c r="C3" s="55" t="s">
         <v>531</v>
       </c>
-      <c r="D3" s="59" t="s">
+      <c r="D3" s="56" t="s">
         <v>532</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="57" t="s">
+      <c r="A4" s="54" t="s">
         <v>59</v>
       </c>
-      <c r="B4" s="57" t="s">
+      <c r="B4" s="54" t="s">
         <v>528</v>
       </c>
-      <c r="C4" s="58" t="s">
+      <c r="C4" s="55" t="s">
         <v>533</v>
       </c>
-      <c r="D4" s="60" t="s">
+      <c r="D4" s="57" t="s">
         <v>534</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="57" t="s">
+      <c r="A5" s="54" t="s">
         <v>71</v>
       </c>
-      <c r="B5" s="57" t="s">
+      <c r="B5" s="54" t="s">
         <v>528</v>
       </c>
-      <c r="C5" s="58" t="s">
+      <c r="C5" s="55" t="s">
         <v>535</v>
       </c>
-      <c r="D5" s="59" t="s">
+      <c r="D5" s="56" t="s">
         <v>536</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="57" t="s">
+      <c r="A6" s="54" t="s">
         <v>73</v>
       </c>
-      <c r="B6" s="57" t="s">
+      <c r="B6" s="54" t="s">
         <v>528</v>
       </c>
-      <c r="C6" s="58" t="s">
+      <c r="C6" s="55" t="s">
         <v>537</v>
       </c>
-      <c r="D6" s="60" t="s">
+      <c r="D6" s="57" t="s">
         <v>538</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="57" t="s">
+      <c r="A7" s="54" t="s">
         <v>75</v>
       </c>
-      <c r="B7" s="57" t="s">
+      <c r="B7" s="54" t="s">
         <v>528</v>
       </c>
-      <c r="C7" s="58" t="s">
+      <c r="C7" s="55" t="s">
         <v>539</v>
       </c>
-      <c r="D7" s="60" t="s">
+      <c r="D7" s="57" t="s">
         <v>540</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="57" t="s">
+      <c r="A8" s="54" t="s">
         <v>67</v>
       </c>
-      <c r="B8" s="57" t="s">
+      <c r="B8" s="54" t="s">
         <v>528</v>
       </c>
-      <c r="C8" s="58" t="s">
+      <c r="C8" s="55" t="s">
         <v>541</v>
       </c>
-      <c r="D8" s="60" t="s">
+      <c r="D8" s="57" t="s">
         <v>542</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="57" t="s">
+      <c r="A9" s="54" t="s">
         <v>57</v>
       </c>
-      <c r="B9" s="57" t="s">
+      <c r="B9" s="54" t="s">
         <v>528</v>
       </c>
-      <c r="C9" s="58" t="s">
+      <c r="C9" s="55" t="s">
         <v>543</v>
       </c>
-      <c r="D9" s="60" t="s">
+      <c r="D9" s="57" t="s">
         <v>544</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="36.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="57" t="s">
+      <c r="A10" s="54" t="s">
         <v>545</v>
       </c>
-      <c r="B10" s="57" t="s">
+      <c r="B10" s="54" t="s">
         <v>528</v>
       </c>
-      <c r="C10" s="61" t="s">
+      <c r="C10" s="58" t="s">
         <v>546</v>
       </c>
-      <c r="D10" s="59" t="s">
+      <c r="D10" s="56" t="s">
         <v>547</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="57" t="s">
+      <c r="A11" s="54" t="s">
         <v>404</v>
       </c>
-      <c r="B11" s="57" t="s">
+      <c r="B11" s="54" t="s">
         <v>528</v>
       </c>
-      <c r="C11" s="58" t="s">
+      <c r="C11" s="55" t="s">
         <v>548</v>
       </c>
-      <c r="D11" s="60" t="s">
+      <c r="D11" s="57" t="s">
         <v>549</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D12" s="62"/>
+      <c r="D12" s="59"/>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="D13" s="62"/>
+      <c r="D13" s="59"/>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -17297,32 +17273,32 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="63" t="s">
+      <c r="A1" s="60" t="s">
         <v>43</v>
       </c>
-      <c r="B1" s="63" t="s">
+      <c r="B1" s="60" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="63" t="s">
+      <c r="A2" s="60" t="s">
         <v>550</v>
       </c>
-      <c r="B2" s="63" t="s">
+      <c r="B2" s="60" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="63" t="s">
+      <c r="A3" s="60" t="s">
         <v>551</v>
       </c>
-      <c r="B3" s="63" t="s">
+      <c r="B3" s="60" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="63"/>
-      <c r="B4" s="63"/>
+      <c r="A4" s="60"/>
+      <c r="B4" s="60"/>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>